<commit_message>
login excel file first row delete
</commit_message>
<xml_diff>
--- a/TestData/login_data.xlsx
+++ b/TestData/login_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ashish_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB4970B1-8B1E-4D88-B473-FA10FCB122CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4161A73-6BEA-47A0-8916-16767C9E2A26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BA1C1957-94B8-4562-BF9E-9BBD605527ED}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
   <si>
     <t>username</t>
   </si>
@@ -49,9 +49,6 @@
   </si>
   <si>
     <t>ashish123</t>
-  </si>
-  <si>
-    <t>success</t>
   </si>
   <si>
     <t>failure</t>
@@ -76,7 +73,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -91,11 +88,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Gadugi"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -119,14 +111,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
@@ -444,7 +430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12987D9E-4E56-427D-98C7-DB61788F7FF0}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
@@ -465,9 +451,9 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
@@ -475,72 +461,60 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>123</v>
       </c>
       <c r="C3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="B4">
         <v>123</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5">
-        <v>123</v>
+      <c r="B5" s="1" t="s">
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{F426C4E1-BEB9-4AA0-B31C-8313BA78AD1D}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{4E54AB48-F77F-447F-9284-32001057332E}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{A302AF30-B1BE-4C08-AF8B-D7F6EE3CBD1A}"/>
-    <hyperlink ref="A5" r:id="rId4" xr:uid="{34935CD0-C32A-4EEF-AE63-5053F1AADCB3}"/>
-    <hyperlink ref="A6" r:id="rId5" xr:uid="{7F0D7A07-6B00-4B4C-868D-FB8DFE4F5952}"/>
-    <hyperlink ref="B6" r:id="rId6" xr:uid="{7F99AB59-662D-4134-982E-6CC098E893DF}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{4E54AB48-F77F-447F-9284-32001057332E}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{A302AF30-B1BE-4C08-AF8B-D7F6EE3CBD1A}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{34935CD0-C32A-4EEF-AE63-5053F1AADCB3}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{7F0D7A07-6B00-4B4C-868D-FB8DFE4F5952}"/>
+    <hyperlink ref="B5" r:id="rId5" xr:uid="{7F99AB59-662D-4134-982E-6CC098E893DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId7"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data add in excel file
</commit_message>
<xml_diff>
--- a/TestData/login_data.xlsx
+++ b/TestData/login_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ashish_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4161A73-6BEA-47A0-8916-16767C9E2A26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89128789-7CAF-4265-ACFF-A1FC4EF51071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BA1C1957-94B8-4562-BF9E-9BBD605527ED}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
   <si>
     <t>username</t>
   </si>
@@ -67,6 +67,9 @@
   </si>
   <si>
     <t>sh@outlook.com</t>
+  </si>
+  <si>
+    <t>success</t>
   </si>
 </sst>
 </file>
@@ -430,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12987D9E-4E56-427D-98C7-DB61788F7FF0}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
@@ -506,6 +509,17 @@
         <v>5</v>
       </c>
     </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{4E54AB48-F77F-447F-9284-32001057332E}"/>
@@ -513,8 +527,9 @@
     <hyperlink ref="A4" r:id="rId3" xr:uid="{34935CD0-C32A-4EEF-AE63-5053F1AADCB3}"/>
     <hyperlink ref="A5" r:id="rId4" xr:uid="{7F0D7A07-6B00-4B4C-868D-FB8DFE4F5952}"/>
     <hyperlink ref="B5" r:id="rId5" xr:uid="{7F99AB59-662D-4134-982E-6CC098E893DF}"/>
+    <hyperlink ref="A8" r:id="rId6" xr:uid="{D0536FA4-C67F-4C10-A99A-919864ED4A8B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update conftest and login data excel file.
</commit_message>
<xml_diff>
--- a/TestData/login_data.xlsx
+++ b/TestData/login_data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ashish_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAA400FC-934C-4371-B7EC-5C2C56F46B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B457DE0-1D7F-4E8A-B9AA-2B181C93DD6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BA1C1957-94B8-4562-BF9E-9BBD605527ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -471,41 +472,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4">
-        <v>123</v>
-      </c>
-      <c r="C4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>5</v>
-      </c>
-    </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
     </row>
@@ -513,11 +479,58 @@
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{4E54AB48-F77F-447F-9284-32001057332E}"/>
     <hyperlink ref="A3" r:id="rId2" xr:uid="{A302AF30-B1BE-4C08-AF8B-D7F6EE3CBD1A}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{34935CD0-C32A-4EEF-AE63-5053F1AADCB3}"/>
-    <hyperlink ref="A5" r:id="rId4" xr:uid="{7F0D7A07-6B00-4B4C-868D-FB8DFE4F5952}"/>
-    <hyperlink ref="B5" r:id="rId5" xr:uid="{7F99AB59-662D-4134-982E-6CC098E893DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5220E0B1-65CB-432D-B8DD-BEC92B99FD5C}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1">
+        <v>123</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{7F99AB59-662D-4134-982E-6CC098E893DF}"/>
+    <hyperlink ref="A2" r:id="rId2" xr:uid="{7F0D7A07-6B00-4B4C-868D-FB8DFE4F5952}"/>
+    <hyperlink ref="A1" r:id="rId3" xr:uid="{34935CD0-C32A-4EEF-AE63-5053F1AADCB3}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>